<commit_message>
Include ECs completed in 2016 in the Value 3BR shortlist
Swap the 10-year age cap for a minimum TOP year (2016), add the eight
ECs that TOP'd in early/mid 2016 (Waterbay, CityLife @ Tampines, Twin
Fountains, The Topiary, Forestville, Lush Acres, SkyPark Residences,
Ecopolitan), and add their matching listings to the shortlist.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBTJbvPDYxoAxHzgUj5que
</commit_message>
<xml_diff>
--- a/output/ec_value_3br_search_snapshot_2026-09-30/shortlist.xlsx
+++ b/output/ec_value_3br_search_snapshot_2026-09-30/shortlist.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,34 +499,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Signature at Yishun</t>
+          <t>Forestville</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2017-07-14</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>9.199999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1098</v>
+        <v>1066</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>1300000</v>
+        <v>1280000</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>1183.97</v>
+        <v>1200.75</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Yishun Street 51</t>
+          <t>38 Woodlands Drive 16</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -536,46 +536,46 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>size matched from search summary</t>
+          <t>older listing ID - may be stale</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-signature-at-yishun-500040599</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-forestville-25455664</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Signature at Yishun</t>
+          <t>Forestville</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2017-07-14</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>9.199999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1098</v>
+        <v>1033</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>1340000</v>
+        <v>1290000</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>1220.4</v>
+        <v>1248.79</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Yishun Street 51</t>
+          <t>22 Woodlands Drive 16</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -583,48 +583,44 @@
       <c r="L3" t="n">
         <v>0</v>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>size matched from search summary</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-signature-at-yishun-500006219</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-forestville-500213788</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Northwave</t>
+          <t>Signature at Yishun</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Yishun</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2019-02-11</t>
+          <t>2017-07-14</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>7.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>1098</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>1360000</v>
+        <v>1300000</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1238.62</v>
+        <v>1183.97</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>111 Woodlands View</t>
+          <t>Yishun Street 51</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -632,44 +628,48 @@
       <c r="L4" t="n">
         <v>0</v>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>size matched from search summary</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-northwave-ec-500112362</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-signature-at-yishun-500040599</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sea Horizon</t>
+          <t>Forestville</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pasir Ris</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2016-10-07</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1098</v>
+        <v>1066</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>1388000</v>
+        <v>1300000</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>1264.12</v>
+        <v>1219.51</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Pasir Ris Rise</t>
+          <t>38 Woodlands Drive 16</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -680,41 +680,41 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500090163</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-forestville-500210303</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sea Horizon</t>
+          <t>Forestville</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pasir Ris</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2016-10-07</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1109</v>
+        <v>1033</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>1400000</v>
+        <v>1300000</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>1262.4</v>
+        <v>1258.47</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>23 Pasir Ris Rise</t>
+          <t>Woodlands Drive 16</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -722,44 +722,48 @@
       <c r="L6" t="n">
         <v>0</v>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>high floor</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500229700</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-forestville-500073495</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>The Criterion</t>
+          <t>Forestville</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2018-02-26</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>8.6</v>
+        <v>10.5</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>1023</v>
+        <v>1087</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>1430000</v>
+        <v>1330000</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>1397.85</v>
+        <v>1223.55</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>7 Yishun Street 51</t>
+          <t>20 Woodlands Drive 16</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -770,14 +774,14 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500212712</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-forestville-500234193</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The Criterion</t>
+          <t>Signature at Yishun</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -787,24 +791,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2018-02-26</t>
+          <t>2017-07-14</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>8.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>1023</v>
+        <v>1098</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>1449999</v>
+        <v>1340000</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>1417.4</v>
+        <v>1220.4</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1 Yishun Street 51</t>
+          <t>Yishun Street 51</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -812,44 +816,48 @@
       <c r="L8" t="n">
         <v>0</v>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>size matched from search summary</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500207742</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-signature-at-yishun-500006219</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sea Horizon</t>
+          <t>Twin Fountains</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pasir Ris</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2016-10-07</t>
+          <t>2016-03-14</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1109</v>
+        <v>1163</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>1450000</v>
+        <v>1360000</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>1307.48</v>
+        <v>1169.39</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>5 Pasir Ris Rise</t>
+          <t>Woodlands Avenue 6</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -857,44 +865,48 @@
       <c r="L9" t="n">
         <v>0</v>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500207797</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-25542447</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>Northwave</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2019-02-11</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8.5</v>
+        <v>7.6</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>1066</v>
+        <v>1098</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>1450000</v>
+        <v>1360000</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>1360.23</v>
+        <v>1238.62</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>33 Sembawang Crescent</t>
+          <t>111 Woodlands View</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -905,41 +917,41 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500158569</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-northwave-ec-500112362</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>The Criterion</t>
+          <t>Twin Fountains</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2018-02-26</t>
+          <t>2016-03-14</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>8.6</v>
+        <v>10.5</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>1033</v>
+        <v>1055</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>1450000</v>
+        <v>1360000</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>1403.68</v>
+        <v>1289.1</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>7 Yishun Street 51</t>
+          <t>Woodlands Avenue 6</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -950,41 +962,41 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500229851</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-500070595</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Westwood Residences</t>
+          <t>Sea Horizon</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Pasir Ris</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2017-10-24</t>
+          <t>2016-10-07</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>8.9</v>
+        <v>10</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1033</v>
+        <v>1098</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>1450000</v>
+        <v>1388000</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>1403.68</v>
+        <v>1264.12</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Westwood Avenue</t>
+          <t>Pasir Ris Rise</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -995,41 +1007,41 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500264493</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500090163</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Westwood Residences</t>
+          <t>Twin Fountains</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2017-10-24</t>
+          <t>2016-03-14</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>8.9</v>
+        <v>10.5</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>1480000</v>
+        <v>1399999</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>1431.33</v>
+        <v>1355.27</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Westwood Avenue</t>
+          <t>Woodlands Avenue 6</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1037,44 +1049,48 @@
       <c r="L13" t="n">
         <v>0</v>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500255283</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60216211</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Bellewoods</t>
+          <t>Sea Horizon</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Pasir Ris</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2017-03-16</t>
+          <t>2016-10-07</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>1066</v>
+        <v>1109</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>1490000</v>
+        <v>1400000</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>1397.75</v>
+        <v>1262.4</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Woodlands Avenue 5</t>
+          <t>23 Pasir Ris Rise</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1085,41 +1101,41 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-bellewoods-500165618</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500229700</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lake Life</t>
+          <t>The Criterion</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Yishun</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2016-12-30</t>
+          <t>2018-02-26</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>9.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>1023</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>1491300</v>
+        <v>1430000</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>1457.77</v>
+        <v>1397.85</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Tao Ching Road</t>
+          <t>7 Yishun Street 51</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1130,41 +1146,41 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-500033581</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500212712</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Westwood Residences</t>
+          <t>The Criterion</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Yishun</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2017-10-24</t>
+          <t>2018-02-26</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>1033</v>
+        <v>1023</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>1498000</v>
+        <v>1449999</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>1450.15</v>
+        <v>1417.4</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Westwood Avenue</t>
+          <t>1 Yishun Street 51</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1175,41 +1191,41 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500276758</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500207742</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>Sea Horizon</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Pasir Ris</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2016-10-07</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1066</v>
+        <v>1109</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>1499999</v>
+        <v>1450000</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>1407.13</v>
+        <v>1307.48</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>25 Sembawang Crescent</t>
+          <t>5 Pasir Ris Rise</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1220,41 +1236,41 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500214081</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500207797</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>The Criterion</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2018-02-26</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1098</v>
+        <v>1066</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>1500000</v>
+        <v>1450000</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>1366.12</v>
+        <v>1360.23</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Yishun Street 51</t>
+          <t>33 Sembawang Crescent</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1262,48 +1278,44 @@
       <c r="L18" t="n">
         <v>0</v>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>high floor; south facing</t>
-        </is>
-      </c>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500107124</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500158569</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Northwave</t>
+          <t>The Criterion</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Yishun</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2019-02-11</t>
+          <t>2018-02-26</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>7.6</v>
+        <v>8.6</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1097</v>
+        <v>1033</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>1500000</v>
+        <v>1450000</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>1367.37</v>
+        <v>1403.68</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Woodlands Avenue 12</t>
+          <t>7 Yishun Street 51</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1311,21 +1323,17 @@
       <c r="L19" t="n">
         <v>0</v>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>older listing ID - may be stale</t>
-        </is>
-      </c>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-northwave-ec-60175231</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500229851</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Lake Life</t>
+          <t>Westwood Residences</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1335,24 +1343,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2016-12-30</t>
+          <t>2017-10-24</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>9.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>1033</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>1500000</v>
+        <v>1450000</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>1452.08</v>
+        <v>1403.68</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2 Tao Ching Road</t>
+          <t>Westwood Avenue</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1360,48 +1368,44 @@
       <c r="L20" t="n">
         <v>0</v>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>older listing ID - may be stale</t>
-        </is>
-      </c>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-25567279</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500264493</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>Twin Fountains</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2016-03-14</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>1066</v>
+        <v>1152</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>1508888</v>
+        <v>1460000</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>1415.47</v>
+        <v>1267.36</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>25 Sembawang Crescent</t>
+          <t>Woodlands Avenue 6</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1409,44 +1413,48 @@
       <c r="L21" t="n">
         <v>0</v>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500073244</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60221142</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>The Amore</t>
+          <t>Westwood Residences</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Jurong West</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2016-11-28</t>
+          <t>2017-10-24</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>9.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1001</v>
+        <v>1034</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>1510000</v>
+        <v>1480000</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>1508.49</v>
+        <v>1431.33</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>53A Edgedale Plains</t>
+          <t>Westwood Avenue</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1454,48 +1462,44 @@
       <c r="L22" t="n">
         <v>0</v>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>older listing ID - may be stale</t>
-        </is>
-      </c>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-amore-24007923</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500255283</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>The Amore</t>
+          <t>Bellewoods</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2016-11-28</t>
+          <t>2017-03-16</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>1001</v>
+        <v>1066</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>1530000</v>
+        <v>1490000</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>1528.47</v>
+        <v>1397.75</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>53 Edgedale Plains</t>
+          <t>Woodlands Avenue 5</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1506,41 +1510,41 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-amore-500196584</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-bellewoods-500165618</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>The Visionaire</t>
+          <t>Lake Life</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Jurong West</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2018-06-14</t>
+          <t>2016-12-30</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>1023</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>1538000</v>
+        <v>1491300</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>1503.42</v>
+        <v>1457.77</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Canberra Drive</t>
+          <t>Tao Ching Road</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1551,41 +1555,41 @@
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-visionaire-500139384</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-500033581</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>Westwood Residences</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Jurong West</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2017-10-24</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>1066</v>
+        <v>1033</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>1548888</v>
+        <v>1498000</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>1452.99</v>
+        <v>1450.15</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>29 Sembawang Crescent</t>
+          <t>Westwood Avenue</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1596,41 +1600,41 @@
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500076102</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500276758</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Westwood Residences</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2017-10-24</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>8.9</v>
+        <v>8.5</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>1033</v>
+        <v>1066</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>1549999</v>
+        <v>1499999</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>1500.48</v>
+        <v>1407.13</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Westwood Avenue</t>
+          <t>25 Sembawang Crescent</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1641,41 +1645,41 @@
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500225608</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500214081</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sea Horizon</t>
+          <t>The Criterion</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Pasir Ris</t>
+          <t>Yishun</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2016-10-07</t>
+          <t>2018-02-26</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>8.6</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>1066</v>
+        <v>1098</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>1550000</v>
+        <v>1500000</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>1454.03</v>
+        <v>1366.12</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>1 Pasir Ris Rise</t>
+          <t>Yishun Street 51</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1683,44 +1687,48 @@
       <c r="L27" t="n">
         <v>0</v>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>high floor; south facing</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500100852</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500107124</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>Northwave</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2019-02-11</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>8.5</v>
+        <v>7.6</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>1109</v>
+        <v>1097</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>1570000</v>
+        <v>1500000</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>1415.69</v>
+        <v>1367.37</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>31 Sembawang Crescent</t>
+          <t>Woodlands Avenue 12</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -1735,7 +1743,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-60080826</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-northwave-ec-60175231</t>
         </is>
       </c>
     </row>
@@ -1759,17 +1767,17 @@
         <v>9.699999999999999</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>1023</v>
+        <v>1033</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>1580000</v>
+        <v>1500000</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>1544.48</v>
+        <v>1452.08</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Tao Ching Road</t>
+          <t>2 Tao Ching Road</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -1784,41 +1792,41 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-60132621</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-25567279</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>The Terrace</t>
+          <t>Forestville</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2017-05-25</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>9.300000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>1001</v>
+        <v>1348</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>1580000</v>
+        <v>1508888</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>1578.42</v>
+        <v>1119.35</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Edgedale Plains</t>
+          <t>Woodlands Drive 16</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -1826,44 +1834,48 @@
       <c r="L30" t="n">
         <v>0</v>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-terrace-500234857</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-forestville-25362802</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>The Terrace</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2017-05-25</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>1001</v>
+        <v>1066</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>1580000</v>
+        <v>1508888</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>1578.42</v>
+        <v>1415.47</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>88 Edgedale Plains</t>
+          <t>25 Sembawang Crescent</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -1871,48 +1883,44 @@
       <c r="L31" t="n">
         <v>0</v>
       </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>same price/size as 500234857 - may be the same unit</t>
-        </is>
-      </c>
+      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-terrace-500138110</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500073244</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Sol Acres</t>
+          <t>The Amore</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Choa Chu Kang</t>
+          <t>Punggol</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2018-03-12</t>
+          <t>2016-11-28</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>8.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>1044</v>
+        <v>1001</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>1599000</v>
+        <v>1510000</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>1531.61</v>
+        <v>1508.49</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Choa Chu Kang Grove</t>
+          <t>53A Edgedale Plains</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
@@ -1920,44 +1928,48 @@
       <c r="L32" t="n">
         <v>0</v>
       </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sol-acres-500267374</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-amore-24007923</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Signature at Yishun</t>
+          <t>The Amore</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Punggol</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2017-07-14</t>
+          <t>2016-11-28</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>9.199999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1098</v>
+        <v>1001</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>1600000</v>
+        <v>1530000</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>1457.19</v>
+        <v>1528.47</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Yishun Street 51</t>
+          <t>53 Edgedale Plains</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
@@ -1965,14 +1977,660 @@
       <c r="L33" t="n">
         <v>0</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-amore-500196584</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>The Visionaire</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Sembawang</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2018-06-14</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>1023</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>1538000</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>1503.42</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Canberra Drive</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-visionaire-500139384</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Parc Life</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Sembawang</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2018-03-29</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>1066</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>1548888</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>1452.99</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>29 Sembawang Crescent</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500076102</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Westwood Residences</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Jurong West</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2017-10-24</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>1033</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>1549999</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>1500.48</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Westwood Avenue</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500225608</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Twin Fountains</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Woodlands</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2016-03-14</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>1152</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>1345.49</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Woodlands Avenue 6</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60107150</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sea Horizon</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Pasir Ris</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2016-10-07</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>10</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>1066</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>1454.03</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>1 Pasir Ris Rise</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500100852</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Parc Life</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sembawang</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2018-03-29</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>1109</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>1570000</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>1415.69</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>31 Sembawang Crescent</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-60080826</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Lake Life</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Jurong West</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2016-12-30</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>1023</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>1580000</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>1544.48</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Tao Ching Road</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-60132621</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>The Terrace</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Punggol</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2017-05-25</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>1001</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>1580000</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>1578.42</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Edgedale Plains</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-terrace-500234857</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>The Terrace</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Punggol</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2017-05-25</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>1001</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>1580000</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>1578.42</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>88 Edgedale Plains</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>same price/size as 500234857 - may be the same unit</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-terrace-500138110</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Twin Fountains</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Woodlands</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2016-03-14</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>1152</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>1588000</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>1378.47</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Woodlands Avenue 6</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-500231540</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Twin Fountains</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Woodlands</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2016-03-14</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>1270</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>1598000</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>1258.27</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Woodlands Avenue 6</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-500211452</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Sol Acres</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Choa Chu Kang</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2018-03-12</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>1044</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>1599000</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>1531.61</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Choa Chu Kang Grove</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sol-acres-500267374</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Signature at Yishun</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Yishun</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2017-07-14</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>1098</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>1457.19</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Yishun Street 51</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="inlineStr">
         <is>
           <t>size matched from search summary</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="N46" t="inlineStr">
         <is>
           <t>https://www.propertyguru.com.sg/listing/for-sale-signature-at-yishun-500275548</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Ecopolitan</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Punggol</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2016-08-29</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>1054</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>1518.03</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Punggol Walk</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-ecopolitan-500222082</t>
         </is>
       </c>
     </row>
@@ -2010,6 +2668,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Crawl each EC project's own PropertyGuru page and report coverage
The Value 3BR run now crawls every eligible project's PropertyGuru page
as well as a keyword search (up to 10 pages each), matches project names
ignoring punctuation (CityLife @ Tampines), and adds a Coverage sheet
with listings seen / in range / kept per project, warning when a project
returns nothing.

Paging now continues while a search keeps returning listings new to that
search, so a keyword search whose first page repeats the project page is
no longer cut short.

Shortlist gains the three Topiary listings June supplied and eight more
found in a second search pass (Parc Life, Sea Horizon, Sol Acres, Twin
Fountains).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBTJbvPDYxoAxHzgUj5que
</commit_message>
<xml_diff>
--- a/output/ec_value_3br_search_snapshot_2026-09-30/shortlist.xlsx
+++ b/output/ec_value_3br_search_snapshot_2026-09-30/shortlist.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -969,34 +969,34 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sea Horizon</t>
+          <t>Twin Fountains</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pasir Ris</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2016-10-07</t>
+          <t>2016-03-14</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1098</v>
+        <v>1055</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>1388000</v>
+        <v>1360000</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>1264.12</v>
+        <v>1289.1</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Pasir Ris Rise</t>
+          <t>11 Woodlands Avenue 6</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1004,44 +1004,48 @@
       <c r="L12" t="n">
         <v>0</v>
       </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>older listing ID; price seen as $1.36M and $1.5M - confirm</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500090163</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60145981</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Twin Fountains</t>
+          <t>Sea Horizon</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Pasir Ris</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2016-03-14</t>
+          <t>2016-10-07</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>1033</v>
+        <v>1098</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>1399999</v>
+        <v>1388000</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>1355.27</v>
+        <v>1264.12</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Woodlands Avenue 6</t>
+          <t>Pasir Ris Rise</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1049,48 +1053,44 @@
       <c r="L13" t="n">
         <v>0</v>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>older listing ID - may be stale</t>
-        </is>
-      </c>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60216211</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500090163</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sea Horizon</t>
+          <t>Twin Fountains</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pasir Ris</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2016-10-07</t>
+          <t>2016-03-14</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>1109</v>
+        <v>1033</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>1400000</v>
+        <v>1399999</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>1262.4</v>
+        <v>1355.27</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>23 Pasir Ris Rise</t>
+          <t>Woodlands Avenue 6</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1098,44 +1098,48 @@
       <c r="L14" t="n">
         <v>0</v>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500229700</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60216211</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>The Criterion</t>
+          <t>Sea Horizon</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Pasir Ris</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2018-02-26</t>
+          <t>2016-10-07</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8.6</v>
+        <v>10</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>1023</v>
+        <v>1109</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>1430000</v>
+        <v>1400000</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>1397.85</v>
+        <v>1262.4</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>7 Yishun Street 51</t>
+          <t>23 Pasir Ris Rise</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1146,7 +1150,7 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500212712</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500229700</t>
         </is>
       </c>
     </row>
@@ -1173,14 +1177,14 @@
         <v>1023</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>1449999</v>
+        <v>1430000</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>1417.4</v>
+        <v>1397.85</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1 Yishun Street 51</t>
+          <t>7 Yishun Street 51</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1191,41 +1195,41 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500207742</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500212712</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sea Horizon</t>
+          <t>The Criterion</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pasir Ris</t>
+          <t>Yishun</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2016-10-07</t>
+          <t>2018-02-26</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>10</v>
+        <v>8.6</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1109</v>
+        <v>1023</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>1450000</v>
+        <v>1449999</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>1307.48</v>
+        <v>1417.4</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>5 Pasir Ris Rise</t>
+          <t>1 Yishun Street 51</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1236,41 +1240,41 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500207797</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500207742</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>Sea Horizon</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Pasir Ris</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2016-10-07</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1066</v>
+        <v>1109</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>1450000</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>1360.23</v>
+        <v>1307.48</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>33 Sembawang Crescent</t>
+          <t>5 Pasir Ris Rise</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1281,41 +1285,41 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500158569</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500207797</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>The Criterion</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2018-02-26</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1033</v>
+        <v>1066</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>1450000</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>1403.68</v>
+        <v>1360.23</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>7 Yishun Street 51</t>
+          <t>33 Sembawang Crescent</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1326,28 +1330,28 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500229851</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500158569</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Westwood Residences</t>
+          <t>The Criterion</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Yishun</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2017-10-24</t>
+          <t>2018-02-26</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>1033</v>
@@ -1360,7 +1364,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Westwood Avenue</t>
+          <t>7 Yishun Street 51</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1371,41 +1375,41 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500264493</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500229851</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Twin Fountains</t>
+          <t>Westwood Residences</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Jurong West</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2016-03-14</t>
+          <t>2017-10-24</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>10.5</v>
+        <v>8.9</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>1152</v>
+        <v>1033</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>1460000</v>
+        <v>1450000</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>1267.36</v>
+        <v>1403.68</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Woodlands Avenue 6</t>
+          <t>Westwood Avenue</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1413,48 +1417,44 @@
       <c r="L21" t="n">
         <v>0</v>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>older listing ID - may be stale</t>
-        </is>
-      </c>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60221142</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500264493</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Westwood Residences</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2017-10-24</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>8.9</v>
+        <v>8.5</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1034</v>
+        <v>1001</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>1480000</v>
+        <v>1450000</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>1431.33</v>
+        <v>1448.55</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Westwood Avenue</t>
+          <t>Sembawang Crescent</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1462,17 +1462,21 @@
       <c r="L22" t="n">
         <v>0</v>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>corner unit</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500255283</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500268300</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bellewoods</t>
+          <t>Twin Fountains</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1482,24 +1486,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2017-03-16</t>
+          <t>2016-03-14</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>1066</v>
+        <v>1152</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>1490000</v>
+        <v>1460000</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>1397.75</v>
+        <v>1267.36</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Woodlands Avenue 5</t>
+          <t>Woodlands Avenue 6</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1507,17 +1511,21 @@
       <c r="L23" t="n">
         <v>0</v>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-bellewoods-500165618</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60221142</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Lake Life</t>
+          <t>Westwood Residences</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1527,24 +1535,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2016-12-30</t>
+          <t>2017-10-24</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1023</v>
+        <v>1034</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>1491300</v>
+        <v>1480000</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>1457.77</v>
+        <v>1431.33</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Tao Ching Road</t>
+          <t>Westwood Avenue</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1555,41 +1563,41 @@
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-500033581</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500255283</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Westwood Residences</t>
+          <t>Bellewoods</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2017-10-24</t>
+          <t>2017-03-16</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>8.9</v>
+        <v>9.5</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>1033</v>
+        <v>1066</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>1498000</v>
+        <v>1490000</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>1450.15</v>
+        <v>1397.75</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Westwood Avenue</t>
+          <t>Woodlands Avenue 5</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1600,41 +1608,41 @@
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500276758</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-bellewoods-500165618</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>Lake Life</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Jurong West</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2016-12-30</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>8.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>1066</v>
+        <v>1023</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>1499999</v>
+        <v>1491300</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>1407.13</v>
+        <v>1457.77</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>25 Sembawang Crescent</t>
+          <t>Tao Ching Road</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1645,41 +1653,41 @@
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500214081</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-500033581</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>The Criterion</t>
+          <t>Westwood Residences</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Jurong West</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2018-02-26</t>
+          <t>2017-10-24</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8.6</v>
+        <v>8.9</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>1098</v>
+        <v>1033</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>1500000</v>
+        <v>1498000</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>1366.12</v>
+        <v>1450.15</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Yishun Street 51</t>
+          <t>Westwood Avenue</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1687,48 +1695,44 @@
       <c r="L27" t="n">
         <v>0</v>
       </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>high floor; south facing</t>
-        </is>
-      </c>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500107124</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500276758</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Northwave</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2019-02-11</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>7.6</v>
+        <v>8.5</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>1097</v>
+        <v>1066</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>1500000</v>
+        <v>1499999</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>1367.37</v>
+        <v>1407.13</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Woodlands Avenue 12</t>
+          <t>25 Sembawang Crescent</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -1736,48 +1740,44 @@
       <c r="L28" t="n">
         <v>0</v>
       </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>older listing ID - may be stale</t>
-        </is>
-      </c>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-northwave-ec-60175231</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500214081</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lake Life</t>
+          <t>The Criterion</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Yishun</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2016-12-30</t>
+          <t>2018-02-26</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>9.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>1033</v>
+        <v>1098</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>1500000</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>1452.08</v>
+        <v>1366.12</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2 Tao Ching Road</t>
+          <t>Yishun Street 51</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -1787,19 +1787,19 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>older listing ID - may be stale</t>
+          <t>high floor; south facing</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-25567279</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-criterion-500107124</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Forestville</t>
+          <t>Northwave</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1809,24 +1809,24 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2016-04-01</t>
+          <t>2019-02-11</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10.5</v>
+        <v>7.6</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>1348</v>
+        <v>1097</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>1508888</v>
+        <v>1500000</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>1119.35</v>
+        <v>1367.37</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Woodlands Drive 16</t>
+          <t>Woodlands Avenue 12</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -1841,41 +1841,41 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-forestville-25362802</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-northwave-ec-60175231</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>Lake Life</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Jurong West</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2016-12-30</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>8.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>1066</v>
+        <v>1033</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>1508888</v>
+        <v>1500000</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>1415.47</v>
+        <v>1452.08</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>25 Sembawang Crescent</t>
+          <t>2 Tao Ching Road</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -1883,44 +1883,48 @@
       <c r="L31" t="n">
         <v>0</v>
       </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500073244</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-25567279</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>The Amore</t>
+          <t>Forestville</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2016-11-28</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>9.800000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>1001</v>
+        <v>1348</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>1510000</v>
+        <v>1508888</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>1508.49</v>
+        <v>1119.35</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>53A Edgedale Plains</t>
+          <t>Woodlands Drive 16</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
@@ -1935,41 +1939,41 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-amore-24007923</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-forestville-25362802</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>The Amore</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2016-11-28</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>9.800000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1001</v>
+        <v>1066</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>1530000</v>
+        <v>1508888</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>1528.47</v>
+        <v>1415.47</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>53 Edgedale Plains</t>
+          <t>25 Sembawang Crescent</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
@@ -1980,41 +1984,41 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-amore-500196584</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500073244</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>The Visionaire</t>
+          <t>The Amore</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Punggol</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2018-06-14</t>
+          <t>2016-11-28</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>8.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>1023</v>
+        <v>1001</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>1538000</v>
+        <v>1510000</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>1503.42</v>
+        <v>1508.49</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Canberra Drive</t>
+          <t>53A Edgedale Plains</t>
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
@@ -2022,44 +2026,48 @@
       <c r="L34" t="n">
         <v>0</v>
       </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-visionaire-500139384</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-amore-24007923</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>The Amore</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Punggol</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2016-11-28</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>8.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>1066</v>
+        <v>1001</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>1548888</v>
+        <v>1530000</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>1452.99</v>
+        <v>1528.47</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>29 Sembawang Crescent</t>
+          <t>53 Edgedale Plains</t>
         </is>
       </c>
       <c r="J35" t="inlineStr"/>
@@ -2070,41 +2078,41 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500076102</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-amore-500196584</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Westwood Residences</t>
+          <t>The Visionaire</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2017-10-24</t>
+          <t>2018-06-14</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>8.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>1033</v>
+        <v>1023</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>1549999</v>
+        <v>1538000</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>1500.48</v>
+        <v>1503.42</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Westwood Avenue</t>
+          <t>Canberra Drive</t>
         </is>
       </c>
       <c r="J36" t="inlineStr"/>
@@ -2115,41 +2123,41 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500225608</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-visionaire-500139384</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Twin Fountains</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2016-03-14</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>1152</v>
+        <v>1066</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>1550000</v>
+        <v>1548888</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>1345.49</v>
+        <v>1452.99</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Woodlands Avenue 6</t>
+          <t>29 Sembawang Crescent</t>
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
@@ -2157,48 +2165,44 @@
       <c r="L37" t="n">
         <v>0</v>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>older listing ID - may be stale</t>
-        </is>
-      </c>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60107150</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500076102</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sea Horizon</t>
+          <t>Westwood Residences</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Pasir Ris</t>
+          <t>Jurong West</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2016-10-07</t>
+          <t>2017-10-24</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>10</v>
+        <v>8.9</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>1066</v>
+        <v>1033</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>1550000</v>
+        <v>1549999</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>1454.03</v>
+        <v>1500.48</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1 Pasir Ris Rise</t>
+          <t>Westwood Avenue</t>
         </is>
       </c>
       <c r="J38" t="inlineStr"/>
@@ -2209,41 +2213,41 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500100852</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-westwood-residences-ec-500225608</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Parc Life</t>
+          <t>Twin Fountains</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Sembawang</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2018-03-29</t>
+          <t>2016-03-14</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>1109</v>
+        <v>1152</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>1570000</v>
+        <v>1550000</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>1415.69</v>
+        <v>1345.49</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>31 Sembawang Crescent</t>
+          <t>Woodlands Avenue 6</t>
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
@@ -2258,41 +2262,41 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-60080826</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-60107150</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Lake Life</t>
+          <t>Sea Horizon</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jurong West</t>
+          <t>Pasir Ris</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2016-12-30</t>
+          <t>2016-10-07</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>9.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>1023</v>
+        <v>1152</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>1580000</v>
+        <v>1550000</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>1544.48</v>
+        <v>1345.49</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Tao Ching Road</t>
+          <t>Pasir Ris Rise</t>
         </is>
       </c>
       <c r="J40" t="inlineStr"/>
@@ -2300,48 +2304,44 @@
       <c r="L40" t="n">
         <v>0</v>
       </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>older listing ID - may be stale</t>
-        </is>
-      </c>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-60132621</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500223553</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>The Terrace</t>
+          <t>Sea Horizon</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Pasir Ris</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2017-05-25</t>
+          <t>2016-10-07</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>9.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>1001</v>
+        <v>1066</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>1580000</v>
+        <v>1550000</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>1578.42</v>
+        <v>1454.03</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Edgedale Plains</t>
+          <t>1 Pasir Ris Rise</t>
         </is>
       </c>
       <c r="J41" t="inlineStr"/>
@@ -2352,41 +2352,41 @@
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-terrace-500234857</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500100852</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>The Terrace</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2017-05-25</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>1001</v>
+        <v>1109</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>1580000</v>
+        <v>1569000</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>1578.42</v>
+        <v>1414.79</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>88 Edgedale Plains</t>
+          <t>Sembawang Crescent</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
@@ -2396,46 +2396,46 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>same price/size as 500234857 - may be the same unit</t>
+          <t>mid floor</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-terrace-500138110</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-500257739</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Twin Fountains</t>
+          <t>Parc Life</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Sembawang</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2016-03-14</t>
+          <t>2018-03-29</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>1152</v>
+        <v>1109</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>1588000</v>
+        <v>1570000</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>1378.47</v>
+        <v>1415.69</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Woodlands Avenue 6</t>
+          <t>31 Sembawang Crescent</t>
         </is>
       </c>
       <c r="J43" t="inlineStr"/>
@@ -2443,44 +2443,48 @@
       <c r="L43" t="n">
         <v>0</v>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-500231540</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-parc-life-60080826</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Twin Fountains</t>
+          <t>Sea Horizon</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Woodlands</t>
+          <t>Pasir Ris</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2016-03-14</t>
+          <t>2016-10-07</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>1270</v>
+        <v>1130</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>1598000</v>
+        <v>1580000</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>1258.27</v>
+        <v>1398.23</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Woodlands Avenue 6</t>
+          <t>Pasir Ris Rise</t>
         </is>
       </c>
       <c r="J44" t="inlineStr"/>
@@ -2491,41 +2495,41 @@
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-500211452</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sea-horizon-500270682</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Sol Acres</t>
+          <t>Lake Life</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Choa Chu Kang</t>
+          <t>Jurong West</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2018-03-12</t>
+          <t>2016-12-30</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1044</v>
+        <v>1023</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>1599000</v>
+        <v>1580000</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>1531.61</v>
+        <v>1544.48</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Choa Chu Kang Grove</t>
+          <t>Tao Ching Road</t>
         </is>
       </c>
       <c r="J45" t="inlineStr"/>
@@ -2533,44 +2537,48 @@
       <c r="L45" t="n">
         <v>0</v>
       </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>older listing ID - may be stale</t>
+        </is>
+      </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-sol-acres-500267374</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-lake-life-60132621</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Signature at Yishun</t>
+          <t>The Terrace</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Punggol</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2017-07-14</t>
+          <t>2017-05-25</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>1098</v>
+        <v>1001</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>1600000</v>
+        <v>1580000</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>1457.19</v>
+        <v>1578.42</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Yishun Street 51</t>
+          <t>Edgedale Plains</t>
         </is>
       </c>
       <c r="J46" t="inlineStr"/>
@@ -2578,21 +2586,17 @@
       <c r="L46" t="n">
         <v>0</v>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>size matched from search summary</t>
-        </is>
-      </c>
+      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-signature-at-yishun-500275548</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-terrace-500234857</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ecopolitan</t>
+          <t>The Terrace</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2602,24 +2606,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2016-08-29</t>
+          <t>2017-05-25</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>10.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>1054</v>
+        <v>1001</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>1600000</v>
+        <v>1580000</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>1518.03</v>
+        <v>1578.42</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Punggol Walk</t>
+          <t>88 Edgedale Plains</t>
         </is>
       </c>
       <c r="J47" t="inlineStr"/>
@@ -2627,10 +2631,439 @@
       <c r="L47" t="n">
         <v>0</v>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>same price/size as 500234857 - may be the same unit</t>
+        </is>
+      </c>
       <c r="N47" t="inlineStr">
         <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-terrace-500138110</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Twin Fountains</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Woodlands</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2016-03-14</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>1152</v>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>1588000</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>1378.47</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Woodlands Avenue 6</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-500231540</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Twin Fountains</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Woodlands</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2016-03-14</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>1270</v>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>1598000</v>
+      </c>
+      <c r="H49" s="3" t="n">
+        <v>1258.27</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Woodlands Avenue 6</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-twin-fountains-500211452</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Sol Acres</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Choa Chu Kang</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2018-03-12</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>1066</v>
+      </c>
+      <c r="G50" s="3" t="n">
+        <v>1599000</v>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Choa Chu Kang Grove</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>low floor; pool view</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sol-acres-500235197</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sol Acres</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Choa Chu Kang</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2018-03-12</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>1044</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>1599000</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>1531.61</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Choa Chu Kang Grove</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-sol-acres-500267374</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Signature at Yishun</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Yishun</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2017-07-14</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>1098</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>1457.19</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Yishun Street 51</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>size matched from search summary</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-signature-at-yishun-500275548</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>The Topiary</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Sengkang</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2016-03-22</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>1087</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>1471.94</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Fernvale Lane</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>price from June's live check 30 Sep; size to confirm</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-topiary-500240724</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>The Topiary</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Sengkang</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2016-03-22</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>1087</v>
+      </c>
+      <c r="G54" s="3" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>1471.94</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>11 Fernvale Lane</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>price from June's live check 30 Sep (search index showed $1.65M)</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-topiary-500104027</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Ecopolitan</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Punggol</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2016-08-29</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>1054</v>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H55" s="3" t="n">
+        <v>1518.03</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Punggol Walk</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr">
+        <is>
           <t>https://www.propertyguru.com.sg/listing/for-sale-ecopolitan-500222082</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>The Topiary</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Sengkang</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2016-03-22</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>1044</v>
+      </c>
+      <c r="G56" s="3" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H56" s="3" t="n">
+        <v>1532.57</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>21 Fernvale Lane</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>from June's links; search index showed $1.638M - confirm price</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-topiary-500229235</t>
         </is>
       </c>
     </row>
@@ -2682,6 +3115,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Let the agent mark a listing's layout, and add Northwave 3 + study
A new optional `layout` column in the shortlist CSV records the agent's
own read of a unit (e.g. "3 + study"). It is shown in the deck and
spreadsheet and overrides the 3-bedroom check, so a unit listed as a
4-bed that is really a 3 + study isn't dropped on the next run.

Adds the 1,270 sqft Northwave patio unit at S$1.6M on that basis.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBTJbvPDYxoAxHzgUj5que
</commit_message>
<xml_diff>
--- a/output/ec_value_3br_search_snapshot_2026-09-30/shortlist.xlsx
+++ b/output/ec_value_3br_search_snapshot_2026-09-30/shortlist.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2829,34 +2829,39 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Signature at Yishun</t>
+          <t>Northwave</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yishun</t>
+          <t>Woodlands</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2017-07-14</t>
+          <t>2019-02-11</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>9.199999999999999</v>
+        <v>7.6</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>3 + study</t>
+        </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>1098</v>
+        <v>1270</v>
       </c>
       <c r="G52" s="3" t="n">
         <v>1600000</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>1457.19</v>
+        <v>1259.84</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Yishun Street 51</t>
+          <t>105 Woodlands View</t>
         </is>
       </c>
       <c r="J52" t="inlineStr"/>
@@ -2866,46 +2871,46 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>size matched from search summary</t>
+          <t>listed as 4-bed; June reads it as 3 + study; pool-facing patio unit; older listing ID</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-signature-at-yishun-500275548</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-northwave-ec-60047599</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>The Topiary</t>
+          <t>Signature at Yishun</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Sengkang</t>
+          <t>Yishun</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2016-03-22</t>
+          <t>2017-07-14</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>10.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>1087</v>
+        <v>1098</v>
       </c>
       <c r="G53" s="3" t="n">
         <v>1600000</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>1471.94</v>
+        <v>1457.19</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Fernvale Lane</t>
+          <t>Yishun Street 51</t>
         </is>
       </c>
       <c r="J53" t="inlineStr"/>
@@ -2915,12 +2920,12 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>price from June's live check 30 Sep; size to confirm</t>
+          <t>size matched from search summary</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-topiary-500240724</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-signature-at-yishun-500275548</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2959,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>11 Fernvale Lane</t>
+          <t>Fernvale Lane</t>
         </is>
       </c>
       <c r="J54" t="inlineStr"/>
@@ -2964,46 +2969,46 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>price from June's live check 30 Sep (search index showed $1.65M)</t>
+          <t>price from June's live check 30 Sep; size to confirm</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-the-topiary-500104027</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-topiary-500240724</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ecopolitan</t>
+          <t>The Topiary</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Punggol</t>
+          <t>Sengkang</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2016-08-29</t>
+          <t>2016-03-22</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>10.1</v>
+        <v>10.5</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>1054</v>
+        <v>1087</v>
       </c>
       <c r="G55" s="3" t="n">
         <v>1600000</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>1518.03</v>
+        <v>1471.94</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Punggol Walk</t>
+          <t>11 Fernvale Lane</t>
         </is>
       </c>
       <c r="J55" t="inlineStr"/>
@@ -3011,44 +3016,48 @@
       <c r="L55" t="n">
         <v>0</v>
       </c>
-      <c r="M55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>price from June's live check 30 Sep (search index showed $1.65M)</t>
+        </is>
+      </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>https://www.propertyguru.com.sg/listing/for-sale-ecopolitan-500222082</t>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-the-topiary-500104027</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>The Topiary</t>
+          <t>Ecopolitan</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Sengkang</t>
+          <t>Punggol</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2016-03-22</t>
+          <t>2016-08-29</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>10.5</v>
+        <v>10.1</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>1044</v>
+        <v>1054</v>
       </c>
       <c r="G56" s="3" t="n">
         <v>1600000</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>1532.57</v>
+        <v>1518.03</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>21 Fernvale Lane</t>
+          <t>Punggol Walk</t>
         </is>
       </c>
       <c r="J56" t="inlineStr"/>
@@ -3056,12 +3065,57 @@
       <c r="L56" t="n">
         <v>0</v>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>https://www.propertyguru.com.sg/listing/for-sale-ecopolitan-500222082</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>The Topiary</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Sengkang</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2016-03-22</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>1044</v>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>1532.57</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>21 Fernvale Lane</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" t="inlineStr">
         <is>
           <t>from June's links; search index showed $1.638M - confirm price</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
+      <c r="N57" t="inlineStr">
         <is>
           <t>https://www.propertyguru.com.sg/listing/for-sale-the-topiary-500229235</t>
         </is>
@@ -3124,6 +3178,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>